<commit_message>
修改 CBReader 目錄之 JA003 = T09n0262_p0056c02 T0262 (卷7) 妙法蓮華經觀世音菩薩普門品
</commit_message>
<xml_diff>
--- a/cbreader2X/nav/simple_nav.xlsx
+++ b/cbreader2X/nav/simple_nav.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cbwork\bin\cbreader2X\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E80152-15A9-4884-9F7C-DB623AA01C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692AA98F-E30A-410B-8EC0-6E8A4A576ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13910,7 +13910,7 @@
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
-    <t>T0262_007 T0262 (卷7) 妙法蓮華經〈觀世音菩薩普門品〉</t>
+    <t>T09n0262_p0056c02 T0262 (卷7) 妙法蓮華經觀世音菩薩普門品</t>
     <phoneticPr fontId="23" type="noConversion"/>
   </si>
 </sst>

</xml_diff>